<commit_message>
Added heat list to the xlsx export https://github.com/daufderheide/racecoordinator_ai/issues/529
</commit_message>
<xml_diff>
--- a/server/src/main/resources/race_export_template.xlsx
+++ b/server/src/main/resources/race_export_template.xlsx
@@ -9,12 +9,67 @@
   <sheets>
     <sheet name="Race Information" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Overall Standings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Heat List" r:id="rId8" sheetId="5"/>
     <sheet name="Heat Template" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Driver Template" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <t>jx:area(lastCell="C5")</t>
+      </text>
+    </comment>
+    <comment ref="A5" authorId="0">
+      <text>
+        <t>jx:each(items="allHeats", var="heat", lastCell="C5")</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="10">
+  <si>
+    <t>Heat List</t>
+  </si>
+  <si>
+    <t>Source: #Section Heat List -&gt; #Table: Heat List</t>
+  </si>
+  <si>
+    <t>Heat</t>
+  </si>
+  <si>
+    <t>Lane 1</t>
+  </si>
+  <si>
+    <t>Lane 2</t>
+  </si>
+  <si>
+    <t>${heat.heatNumber}</t>
+  </si>
+  <si>
+    <t>${heat.drivers[0].actualDriver.name}</t>
+  </si>
+  <si>
+    <t>${heat.drivers[1].actualDriver.name}</t>
+  </si>
+  <si>
+    <t>${heat.getDriverNameOnLane(0)}</t>
+  </si>
+  <si>
+    <t>${heat.getDriverNameOnLane(1)}</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -241,6 +296,10 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -535,8 +594,8 @@
   <dimension ref="A1:B81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col min="1" max="1" customWidth="true" width="38.0"/>
+    <col min="2" max="2" customWidth="true" width="95.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1453,17 +1512,17 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col min="1" max="1" customWidth="true" width="13.0"/>
+    <col min="2" max="2" customWidth="true" width="45.0"/>
+    <col min="3" max="3" customWidth="true" width="13.0"/>
+    <col min="4" max="4" customWidth="true" width="13.0"/>
+    <col min="5" max="5" customWidth="true" width="14.0"/>
+    <col min="6" max="6" customWidth="true" width="14.0"/>
+    <col min="7" max="7" customWidth="true" width="16.0"/>
+    <col min="8" max="8" customWidth="true" width="19.0"/>
+    <col min="9" max="9" customWidth="true" width="18.0"/>
+    <col min="10" max="10" customWidth="true" width="16.0"/>
+    <col min="11" max="11" customWidth="true" width="18.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1609,15 +1668,15 @@
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col min="1" max="1" customWidth="true" width="55.0"/>
+    <col min="2" max="2" customWidth="true" width="12.0"/>
+    <col min="3" max="3" customWidth="true" width="13.0"/>
+    <col min="4" max="4" customWidth="true" width="13.0"/>
+    <col min="5" max="5" customWidth="true" width="16.0"/>
+    <col min="6" max="6" customWidth="true" width="19.0"/>
+    <col min="7" max="7" customWidth="true" width="18.0"/>
+    <col min="8" max="8" customWidth="true" width="16.0"/>
+    <col min="9" max="9" customWidth="true" width="18.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1743,10 +1802,10 @@
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="85" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="85.0"/>
+    <col min="2" max="2" customWidth="true" width="21.0"/>
+    <col min="3" max="3" customWidth="true" width="21.0"/>
+    <col min="4" max="4" customWidth="true" width="12.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1923,4 +1982,48 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <legacyDrawing r:id="rId15"/>
+</worksheet>
 </file>
</xml_diff>